<commit_message>
Add Android App Build & Test workflow (build-android -> appium-report DAG)
</commit_message>
<xml_diff>
--- a/Appium_Mobile_300_Test_Report.xlsx
+++ b/Appium_Mobile_300_Test_Report.xlsx
@@ -979,7 +979,7 @@
       </c>
       <c r="H2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I2" s="15" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H3" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I3" s="15" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="H5" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="H8" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I9" s="15" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="H10" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I10" s="15" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I11" s="15" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I12" s="15" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="H13" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I13" s="15" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I14" s="15" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I15" s="15" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="H16" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I16" s="15" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="H18" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I18" s="15" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I19" s="15" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I20" s="15" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I21" s="15" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I22" s="15" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I23" s="15" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I24" s="15" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I25" s="15" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I26" s="15" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="H27" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I27" s="15" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="H28" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I28" s="15" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="H29" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I29" s="15" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="H30" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I30" s="15" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I31" s="15" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I32" s="15" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I33" s="15" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="H34" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I34" s="15" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I35" s="15" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I36" s="15" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="H37" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I37" s="15" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="H38" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I38" s="15" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="H39" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I39" s="15" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="H40" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I40" s="15" t="inlineStr">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="H41" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I41" s="15" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="H42" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I42" s="15" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="H43" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I43" s="15" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="H44" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I44" s="15" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="H45" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I45" s="15" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="H46" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I46" s="15" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="H47" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I47" s="15" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="H48" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I48" s="15" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="H49" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I49" s="15" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="H50" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I50" s="15" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="H51" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I51" s="15" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="H52" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I52" s="15" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="H53" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I53" s="15" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="H54" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I54" s="15" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="H55" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I55" s="15" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="H56" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I56" s="15" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="H57" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I57" s="15" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="H58" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I58" s="15" t="inlineStr">
@@ -3544,7 +3544,7 @@
       </c>
       <c r="H59" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I59" s="15" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="H60" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I60" s="15" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="H61" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I61" s="15" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="H62" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I62" s="15" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="H63" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I63" s="15" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="H64" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I64" s="15" t="inlineStr">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="H65" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I65" s="15" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="H66" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I66" s="15" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="H67" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I67" s="15" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="H68" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I68" s="15" t="inlineStr">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="H69" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I69" s="15" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="H70" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I70" s="15" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="H71" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I71" s="15" t="inlineStr">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="H72" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I72" s="15" t="inlineStr">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="H73" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I73" s="15" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="H74" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I74" s="15" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="H75" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I75" s="15" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="H76" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I76" s="15" t="inlineStr">
@@ -4354,7 +4354,7 @@
       </c>
       <c r="H77" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I77" s="15" t="inlineStr">
@@ -4395,11 +4395,11 @@
         </is>
       </c>
       <c r="G78" s="17" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="H78" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I78" s="15" t="inlineStr">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="H79" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I79" s="15" t="inlineStr">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="H80" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I80" s="15" t="inlineStr">
@@ -4534,7 +4534,7 @@
       </c>
       <c r="H81" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I81" s="15" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="H82" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I82" s="15" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="H83" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I83" s="15" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="H84" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I84" s="15" t="inlineStr">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="H85" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I85" s="15" t="inlineStr">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="H86" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I86" s="15" t="inlineStr">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="H87" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I87" s="15" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="H88" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I88" s="15" t="inlineStr">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="H89" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I89" s="15" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="H90" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I90" s="15" t="inlineStr">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="H91" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I91" s="15" t="inlineStr">
@@ -5029,7 +5029,7 @@
       </c>
       <c r="H92" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I92" s="15" t="inlineStr">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="H93" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I93" s="15" t="inlineStr">
@@ -5119,7 +5119,7 @@
       </c>
       <c r="H94" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I94" s="15" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="H95" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I95" s="15" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="H96" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I96" s="15" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H97" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I97" s="15" t="inlineStr">
@@ -5299,7 +5299,7 @@
       </c>
       <c r="H98" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I98" s="15" t="inlineStr">
@@ -5344,7 +5344,7 @@
       </c>
       <c r="H99" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I99" s="15" t="inlineStr">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="H100" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I100" s="15" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="H101" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I101" s="15" t="inlineStr">
@@ -5479,7 +5479,7 @@
       </c>
       <c r="H102" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I102" s="15" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="H103" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I103" s="15" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="H104" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I104" s="15" t="inlineStr">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="H105" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I105" s="15" t="inlineStr">
@@ -5659,7 +5659,7 @@
       </c>
       <c r="H106" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I106" s="15" t="inlineStr">
@@ -5704,7 +5704,7 @@
       </c>
       <c r="H107" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I107" s="15" t="inlineStr">
@@ -5749,7 +5749,7 @@
       </c>
       <c r="H108" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I108" s="15" t="inlineStr">
@@ -5794,7 +5794,7 @@
       </c>
       <c r="H109" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I109" s="15" t="inlineStr">
@@ -5839,7 +5839,7 @@
       </c>
       <c r="H110" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I110" s="15" t="inlineStr">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="H111" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I111" s="15" t="inlineStr">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="H112" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I112" s="15" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="H113" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I113" s="15" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="H114" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I114" s="15" t="inlineStr">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="H115" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I115" s="15" t="inlineStr">
@@ -6109,7 +6109,7 @@
       </c>
       <c r="H116" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I116" s="15" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="H117" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I117" s="15" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="H118" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I118" s="15" t="inlineStr">
@@ -6244,7 +6244,7 @@
       </c>
       <c r="H119" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I119" s="15" t="inlineStr">
@@ -6289,7 +6289,7 @@
       </c>
       <c r="H120" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I120" s="15" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="H121" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I121" s="15" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="H122" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I122" s="15" t="inlineStr">
@@ -6424,7 +6424,7 @@
       </c>
       <c r="H123" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I123" s="15" t="inlineStr">
@@ -6469,7 +6469,7 @@
       </c>
       <c r="H124" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I124" s="15" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="H125" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I125" s="15" t="inlineStr">
@@ -6559,7 +6559,7 @@
       </c>
       <c r="H126" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I126" s="15" t="inlineStr">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="H127" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I127" s="15" t="inlineStr">
@@ -6649,7 +6649,7 @@
       </c>
       <c r="H128" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I128" s="15" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="H129" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I129" s="15" t="inlineStr">
@@ -6739,7 +6739,7 @@
       </c>
       <c r="H130" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I130" s="15" t="inlineStr">
@@ -6784,7 +6784,7 @@
       </c>
       <c r="H131" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I131" s="15" t="inlineStr">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="H132" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I132" s="15" t="inlineStr">
@@ -6874,7 +6874,7 @@
       </c>
       <c r="H133" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I133" s="15" t="inlineStr">
@@ -6919,7 +6919,7 @@
       </c>
       <c r="H134" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I134" s="15" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="H135" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I135" s="15" t="inlineStr">
@@ -7009,7 +7009,7 @@
       </c>
       <c r="H136" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I136" s="15" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="H137" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I137" s="15" t="inlineStr">
@@ -7099,7 +7099,7 @@
       </c>
       <c r="H138" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I138" s="15" t="inlineStr">
@@ -7144,7 +7144,7 @@
       </c>
       <c r="H139" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I139" s="15" t="inlineStr">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="H140" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I140" s="15" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="H141" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I141" s="15" t="inlineStr">
@@ -7279,7 +7279,7 @@
       </c>
       <c r="H142" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I142" s="15" t="inlineStr">
@@ -7324,7 +7324,7 @@
       </c>
       <c r="H143" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I143" s="15" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="H144" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I144" s="15" t="inlineStr">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="H145" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I145" s="15" t="inlineStr">
@@ -7459,7 +7459,7 @@
       </c>
       <c r="H146" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I146" s="15" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="H147" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I147" s="15" t="inlineStr">
@@ -7549,7 +7549,7 @@
       </c>
       <c r="H148" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I148" s="15" t="inlineStr">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="H149" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I149" s="15" t="inlineStr">
@@ -7639,7 +7639,7 @@
       </c>
       <c r="H150" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I150" s="15" t="inlineStr">
@@ -7684,7 +7684,7 @@
       </c>
       <c r="H151" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I151" s="15" t="inlineStr">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="H152" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I152" s="15" t="inlineStr">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="H153" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I153" s="15" t="inlineStr">
@@ -7819,7 +7819,7 @@
       </c>
       <c r="H154" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I154" s="15" t="inlineStr">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="H155" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I155" s="15" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="H156" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I156" s="15" t="inlineStr">
@@ -7954,7 +7954,7 @@
       </c>
       <c r="H157" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I157" s="15" t="inlineStr">
@@ -7999,7 +7999,7 @@
       </c>
       <c r="H158" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I158" s="15" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="H159" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I159" s="15" t="inlineStr">
@@ -8089,7 +8089,7 @@
       </c>
       <c r="H160" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I160" s="15" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H161" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I161" s="15" t="inlineStr">
@@ -8179,7 +8179,7 @@
       </c>
       <c r="H162" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I162" s="15" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="H163" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I163" s="15" t="inlineStr">
@@ -8269,7 +8269,7 @@
       </c>
       <c r="H164" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I164" s="15" t="inlineStr">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="H165" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I165" s="15" t="inlineStr">
@@ -8359,7 +8359,7 @@
       </c>
       <c r="H166" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I166" s="15" t="inlineStr">
@@ -8404,7 +8404,7 @@
       </c>
       <c r="H167" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I167" s="15" t="inlineStr">
@@ -8449,7 +8449,7 @@
       </c>
       <c r="H168" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I168" s="15" t="inlineStr">
@@ -8494,7 +8494,7 @@
       </c>
       <c r="H169" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I169" s="15" t="inlineStr">
@@ -8539,7 +8539,7 @@
       </c>
       <c r="H170" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I170" s="15" t="inlineStr">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H171" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I171" s="15" t="inlineStr">
@@ -8629,7 +8629,7 @@
       </c>
       <c r="H172" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I172" s="15" t="inlineStr">
@@ -8674,7 +8674,7 @@
       </c>
       <c r="H173" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I173" s="15" t="inlineStr">
@@ -8719,7 +8719,7 @@
       </c>
       <c r="H174" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I174" s="15" t="inlineStr">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="H175" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I175" s="15" t="inlineStr">
@@ -8809,7 +8809,7 @@
       </c>
       <c r="H176" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I176" s="15" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="H177" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I177" s="15" t="inlineStr">
@@ -8899,7 +8899,7 @@
       </c>
       <c r="H178" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I178" s="15" t="inlineStr">
@@ -8944,7 +8944,7 @@
       </c>
       <c r="H179" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I179" s="15" t="inlineStr">
@@ -8989,7 +8989,7 @@
       </c>
       <c r="H180" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I180" s="15" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="H181" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I181" s="15" t="inlineStr">
@@ -9079,7 +9079,7 @@
       </c>
       <c r="H182" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I182" s="15" t="inlineStr">
@@ -9124,7 +9124,7 @@
       </c>
       <c r="H183" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I183" s="15" t="inlineStr">
@@ -9169,7 +9169,7 @@
       </c>
       <c r="H184" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I184" s="15" t="inlineStr">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="H185" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I185" s="15" t="inlineStr">
@@ -9259,7 +9259,7 @@
       </c>
       <c r="H186" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I186" s="15" t="inlineStr">
@@ -9304,7 +9304,7 @@
       </c>
       <c r="H187" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I187" s="15" t="inlineStr">
@@ -9349,7 +9349,7 @@
       </c>
       <c r="H188" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I188" s="15" t="inlineStr">
@@ -9394,7 +9394,7 @@
       </c>
       <c r="H189" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I189" s="15" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="H190" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I190" s="15" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="H191" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I191" s="15" t="inlineStr">
@@ -9529,7 +9529,7 @@
       </c>
       <c r="H192" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I192" s="15" t="inlineStr">
@@ -9574,7 +9574,7 @@
       </c>
       <c r="H193" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I193" s="15" t="inlineStr">
@@ -9619,7 +9619,7 @@
       </c>
       <c r="H194" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I194" s="15" t="inlineStr">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="H195" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I195" s="15" t="inlineStr">
@@ -9709,7 +9709,7 @@
       </c>
       <c r="H196" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I196" s="15" t="inlineStr">
@@ -9754,7 +9754,7 @@
       </c>
       <c r="H197" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I197" s="15" t="inlineStr">
@@ -9799,7 +9799,7 @@
       </c>
       <c r="H198" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I198" s="15" t="inlineStr">
@@ -9844,7 +9844,7 @@
       </c>
       <c r="H199" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I199" s="15" t="inlineStr">
@@ -9889,7 +9889,7 @@
       </c>
       <c r="H200" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I200" s="15" t="inlineStr">
@@ -9934,7 +9934,7 @@
       </c>
       <c r="H201" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I201" s="15" t="inlineStr">
@@ -9979,7 +9979,7 @@
       </c>
       <c r="H202" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I202" s="15" t="inlineStr">
@@ -10024,7 +10024,7 @@
       </c>
       <c r="H203" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I203" s="15" t="inlineStr">
@@ -10069,7 +10069,7 @@
       </c>
       <c r="H204" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I204" s="15" t="inlineStr">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="H205" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I205" s="15" t="inlineStr">
@@ -10159,7 +10159,7 @@
       </c>
       <c r="H206" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I206" s="15" t="inlineStr">
@@ -10204,7 +10204,7 @@
       </c>
       <c r="H207" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I207" s="15" t="inlineStr">
@@ -10249,7 +10249,7 @@
       </c>
       <c r="H208" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I208" s="15" t="inlineStr">
@@ -10294,7 +10294,7 @@
       </c>
       <c r="H209" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I209" s="15" t="inlineStr">
@@ -10339,7 +10339,7 @@
       </c>
       <c r="H210" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I210" s="15" t="inlineStr">
@@ -10384,7 +10384,7 @@
       </c>
       <c r="H211" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I211" s="15" t="inlineStr">
@@ -10429,7 +10429,7 @@
       </c>
       <c r="H212" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I212" s="15" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="H213" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I213" s="15" t="inlineStr">
@@ -10519,7 +10519,7 @@
       </c>
       <c r="H214" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I214" s="15" t="inlineStr">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="H215" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I215" s="15" t="inlineStr">
@@ -10609,7 +10609,7 @@
       </c>
       <c r="H216" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I216" s="15" t="inlineStr">
@@ -10654,7 +10654,7 @@
       </c>
       <c r="H217" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I217" s="15" t="inlineStr">
@@ -10699,7 +10699,7 @@
       </c>
       <c r="H218" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I218" s="15" t="inlineStr">
@@ -10744,7 +10744,7 @@
       </c>
       <c r="H219" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I219" s="15" t="inlineStr">
@@ -10789,7 +10789,7 @@
       </c>
       <c r="H220" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I220" s="15" t="inlineStr">
@@ -10834,7 +10834,7 @@
       </c>
       <c r="H221" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I221" s="15" t="inlineStr">
@@ -10879,7 +10879,7 @@
       </c>
       <c r="H222" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I222" s="15" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="H223" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I223" s="15" t="inlineStr">
@@ -10969,7 +10969,7 @@
       </c>
       <c r="H224" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I224" s="15" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H225" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I225" s="15" t="inlineStr">
@@ -11059,7 +11059,7 @@
       </c>
       <c r="H226" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I226" s="15" t="inlineStr">
@@ -11104,7 +11104,7 @@
       </c>
       <c r="H227" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I227" s="15" t="inlineStr">
@@ -11149,7 +11149,7 @@
       </c>
       <c r="H228" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I228" s="15" t="inlineStr">
@@ -11194,7 +11194,7 @@
       </c>
       <c r="H229" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I229" s="15" t="inlineStr">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="H230" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I230" s="15" t="inlineStr">
@@ -11284,7 +11284,7 @@
       </c>
       <c r="H231" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I231" s="15" t="inlineStr">
@@ -11329,7 +11329,7 @@
       </c>
       <c r="H232" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I232" s="15" t="inlineStr">
@@ -11374,7 +11374,7 @@
       </c>
       <c r="H233" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I233" s="15" t="inlineStr">
@@ -11419,7 +11419,7 @@
       </c>
       <c r="H234" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I234" s="15" t="inlineStr">
@@ -11464,7 +11464,7 @@
       </c>
       <c r="H235" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I235" s="15" t="inlineStr">
@@ -11509,7 +11509,7 @@
       </c>
       <c r="H236" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I236" s="15" t="inlineStr">
@@ -11554,7 +11554,7 @@
       </c>
       <c r="H237" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I237" s="15" t="inlineStr">
@@ -11599,7 +11599,7 @@
       </c>
       <c r="H238" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I238" s="15" t="inlineStr">
@@ -11644,7 +11644,7 @@
       </c>
       <c r="H239" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I239" s="15" t="inlineStr">
@@ -11689,7 +11689,7 @@
       </c>
       <c r="H240" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I240" s="15" t="inlineStr">
@@ -11734,7 +11734,7 @@
       </c>
       <c r="H241" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I241" s="15" t="inlineStr">
@@ -11779,7 +11779,7 @@
       </c>
       <c r="H242" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I242" s="15" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="H243" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I243" s="15" t="inlineStr">
@@ -11869,7 +11869,7 @@
       </c>
       <c r="H244" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I244" s="15" t="inlineStr">
@@ -11914,7 +11914,7 @@
       </c>
       <c r="H245" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I245" s="15" t="inlineStr">
@@ -11959,7 +11959,7 @@
       </c>
       <c r="H246" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I246" s="15" t="inlineStr">
@@ -12004,7 +12004,7 @@
       </c>
       <c r="H247" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I247" s="15" t="inlineStr">
@@ -12049,7 +12049,7 @@
       </c>
       <c r="H248" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I248" s="15" t="inlineStr">
@@ -12094,7 +12094,7 @@
       </c>
       <c r="H249" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I249" s="15" t="inlineStr">
@@ -12139,7 +12139,7 @@
       </c>
       <c r="H250" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I250" s="15" t="inlineStr">
@@ -12184,7 +12184,7 @@
       </c>
       <c r="H251" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I251" s="15" t="inlineStr">
@@ -12229,7 +12229,7 @@
       </c>
       <c r="H252" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I252" s="15" t="inlineStr">
@@ -12274,7 +12274,7 @@
       </c>
       <c r="H253" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I253" s="15" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="H254" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I254" s="15" t="inlineStr">
@@ -12364,7 +12364,7 @@
       </c>
       <c r="H255" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I255" s="15" t="inlineStr">
@@ -12409,7 +12409,7 @@
       </c>
       <c r="H256" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I256" s="15" t="inlineStr">
@@ -12454,7 +12454,7 @@
       </c>
       <c r="H257" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I257" s="15" t="inlineStr">
@@ -12499,7 +12499,7 @@
       </c>
       <c r="H258" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I258" s="15" t="inlineStr">
@@ -12544,7 +12544,7 @@
       </c>
       <c r="H259" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I259" s="15" t="inlineStr">
@@ -12589,7 +12589,7 @@
       </c>
       <c r="H260" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I260" s="15" t="inlineStr">
@@ -12634,7 +12634,7 @@
       </c>
       <c r="H261" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I261" s="15" t="inlineStr">
@@ -12679,7 +12679,7 @@
       </c>
       <c r="H262" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I262" s="15" t="inlineStr">
@@ -12724,7 +12724,7 @@
       </c>
       <c r="H263" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I263" s="15" t="inlineStr">
@@ -12769,7 +12769,7 @@
       </c>
       <c r="H264" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I264" s="15" t="inlineStr">
@@ -12814,7 +12814,7 @@
       </c>
       <c r="H265" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I265" s="15" t="inlineStr">
@@ -12859,7 +12859,7 @@
       </c>
       <c r="H266" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I266" s="15" t="inlineStr">
@@ -12904,7 +12904,7 @@
       </c>
       <c r="H267" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I267" s="15" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="H268" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I268" s="15" t="inlineStr">
@@ -12994,7 +12994,7 @@
       </c>
       <c r="H269" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I269" s="15" t="inlineStr">
@@ -13039,7 +13039,7 @@
       </c>
       <c r="H270" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I270" s="15" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="H271" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I271" s="15" t="inlineStr">
@@ -13129,7 +13129,7 @@
       </c>
       <c r="H272" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I272" s="15" t="inlineStr">
@@ -13174,7 +13174,7 @@
       </c>
       <c r="H273" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I273" s="15" t="inlineStr">
@@ -13219,7 +13219,7 @@
       </c>
       <c r="H274" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I274" s="15" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="H275" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I275" s="15" t="inlineStr">
@@ -13309,7 +13309,7 @@
       </c>
       <c r="H276" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I276" s="15" t="inlineStr">
@@ -13354,7 +13354,7 @@
       </c>
       <c r="H277" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I277" s="15" t="inlineStr">
@@ -13399,7 +13399,7 @@
       </c>
       <c r="H278" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I278" s="15" t="inlineStr">
@@ -13444,7 +13444,7 @@
       </c>
       <c r="H279" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I279" s="15" t="inlineStr">
@@ -13489,7 +13489,7 @@
       </c>
       <c r="H280" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I280" s="15" t="inlineStr">
@@ -13534,7 +13534,7 @@
       </c>
       <c r="H281" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I281" s="15" t="inlineStr">
@@ -13579,7 +13579,7 @@
       </c>
       <c r="H282" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I282" s="15" t="inlineStr">
@@ -13624,7 +13624,7 @@
       </c>
       <c r="H283" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I283" s="15" t="inlineStr">
@@ -13669,7 +13669,7 @@
       </c>
       <c r="H284" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I284" s="15" t="inlineStr">
@@ -13714,7 +13714,7 @@
       </c>
       <c r="H285" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I285" s="15" t="inlineStr">
@@ -13759,7 +13759,7 @@
       </c>
       <c r="H286" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I286" s="15" t="inlineStr">
@@ -13804,7 +13804,7 @@
       </c>
       <c r="H287" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I287" s="15" t="inlineStr">
@@ -13849,7 +13849,7 @@
       </c>
       <c r="H288" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I288" s="15" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H289" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I289" s="15" t="inlineStr">
@@ -13939,7 +13939,7 @@
       </c>
       <c r="H290" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I290" s="15" t="inlineStr">
@@ -13984,7 +13984,7 @@
       </c>
       <c r="H291" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I291" s="15" t="inlineStr">
@@ -14029,7 +14029,7 @@
       </c>
       <c r="H292" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I292" s="15" t="inlineStr">
@@ -14074,7 +14074,7 @@
       </c>
       <c r="H293" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I293" s="15" t="inlineStr">
@@ -14119,7 +14119,7 @@
       </c>
       <c r="H294" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I294" s="15" t="inlineStr">
@@ -14164,7 +14164,7 @@
       </c>
       <c r="H295" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I295" s="15" t="inlineStr">
@@ -14209,7 +14209,7 @@
       </c>
       <c r="H296" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I296" s="15" t="inlineStr">
@@ -14254,7 +14254,7 @@
       </c>
       <c r="H297" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I297" s="15" t="inlineStr">
@@ -14299,7 +14299,7 @@
       </c>
       <c r="H298" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I298" s="15" t="inlineStr">
@@ -14344,7 +14344,7 @@
       </c>
       <c r="H299" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I299" s="15" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="H300" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I300" s="15" t="inlineStr">
@@ -14434,7 +14434,7 @@
       </c>
       <c r="H301" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07 10:16:39</t>
+          <t>2026-08-07 11:33:28</t>
         </is>
       </c>
       <c r="I301" s="15" t="inlineStr">

</xml_diff>